<commit_message>
se arreglan perfiles como biometria
</commit_message>
<xml_diff>
--- a/observations-summary.xlsx
+++ b/observations-summary.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="88">
   <si>
     <t>Profile</t>
   </si>
@@ -159,6 +159,12 @@
   </si>
   <si>
     <t>SNOMED CT#41633001</t>
+  </si>
+  <si>
+    <t>iol-formula-result</t>
+  </si>
+  <si>
+    <t>IOL Formula Result</t>
   </si>
   <si>
     <t>krimsky-test</t>
@@ -4524,7 +4530,7 @@
         <v>16</v>
       </c>
       <c r="H118" t="s" s="2">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="I118" t="s" s="2">
         <v>18</v>
@@ -4608,13 +4614,13 @@
     </row>
     <row r="121">
       <c r="A121" t="s" s="2">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="B121" t="s" s="2">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C121" t="s" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D121" t="s" s="2">
         <v>14</v>
@@ -4623,13 +4629,13 @@
         <v>14</v>
       </c>
       <c r="F121" t="s" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G121" t="s" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H121" t="s" s="2">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="I121" t="s" s="2">
         <v>18</v>
@@ -4643,13 +4649,13 @@
     </row>
     <row r="122">
       <c r="A122" t="s" s="2">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="B122" t="s" s="2">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C122" t="s" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D122" t="s" s="2">
         <v>14</v>
@@ -4658,13 +4664,13 @@
         <v>14</v>
       </c>
       <c r="F122" t="s" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G122" t="s" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H122" t="s" s="2">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I122" t="s" s="2">
         <v>18</v>
@@ -4681,7 +4687,7 @@
         <v>14</v>
       </c>
       <c r="B123" t="s" s="2">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C123" t="s" s="2">
         <v>14</v>
@@ -4699,7 +4705,7 @@
         <v>14</v>
       </c>
       <c r="H123" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I123" t="s" s="2">
         <v>18</v>
@@ -4716,7 +4722,7 @@
         <v>14</v>
       </c>
       <c r="B124" t="s" s="2">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C124" t="s" s="2">
         <v>14</v>
@@ -4734,7 +4740,7 @@
         <v>14</v>
       </c>
       <c r="H124" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I124" t="s" s="2">
         <v>18</v>
@@ -4748,13 +4754,13 @@
     </row>
     <row r="125">
       <c r="A125" t="s" s="2">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="B125" t="s" s="2">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C125" t="s" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D125" t="s" s="2">
         <v>14</v>
@@ -4763,13 +4769,13 @@
         <v>14</v>
       </c>
       <c r="F125" t="s" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G125" t="s" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H125" t="s" s="2">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I125" t="s" s="2">
         <v>18</v>
@@ -4783,13 +4789,13 @@
     </row>
     <row r="126">
       <c r="A126" t="s" s="2">
-        <v>14</v>
+        <v>51</v>
       </c>
       <c r="B126" t="s" s="2">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C126" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D126" t="s" s="2">
         <v>14</v>
@@ -4798,13 +4804,13 @@
         <v>14</v>
       </c>
       <c r="F126" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G126" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H126" t="s" s="2">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="I126" t="s" s="2">
         <v>18</v>
@@ -4821,7 +4827,7 @@
         <v>14</v>
       </c>
       <c r="B127" t="s" s="2">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C127" t="s" s="2">
         <v>14</v>
@@ -4839,7 +4845,7 @@
         <v>14</v>
       </c>
       <c r="H127" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I127" t="s" s="2">
         <v>18</v>
@@ -4856,7 +4862,7 @@
         <v>14</v>
       </c>
       <c r="B128" t="s" s="2">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C128" t="s" s="2">
         <v>14</v>
@@ -4874,7 +4880,7 @@
         <v>14</v>
       </c>
       <c r="H128" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I128" t="s" s="2">
         <v>18</v>
@@ -4888,13 +4894,13 @@
     </row>
     <row r="129">
       <c r="A129" t="s" s="2">
-        <v>14</v>
+        <v>53</v>
       </c>
       <c r="B129" t="s" s="2">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C129" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D129" t="s" s="2">
         <v>14</v>
@@ -4903,13 +4909,13 @@
         <v>14</v>
       </c>
       <c r="F129" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G129" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H129" t="s" s="2">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="I129" t="s" s="2">
         <v>18</v>
@@ -4923,13 +4929,13 @@
     </row>
     <row r="130">
       <c r="A130" t="s" s="2">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="B130" t="s" s="2">
         <v>57</v>
       </c>
       <c r="C130" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D130" t="s" s="2">
         <v>14</v>
@@ -4938,13 +4944,13 @@
         <v>14</v>
       </c>
       <c r="F130" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G130" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H130" t="s" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I130" t="s" s="2">
         <v>18</v>
@@ -5028,13 +5034,13 @@
     </row>
     <row r="133">
       <c r="A133" t="s" s="2">
-        <v>14</v>
+        <v>58</v>
       </c>
       <c r="B133" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C133" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D133" t="s" s="2">
         <v>14</v>
@@ -5043,13 +5049,13 @@
         <v>14</v>
       </c>
       <c r="F133" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G133" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H133" t="s" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I133" t="s" s="2">
         <v>18</v>
@@ -5066,7 +5072,7 @@
         <v>14</v>
       </c>
       <c r="B134" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C134" t="s" s="2">
         <v>14</v>
@@ -5084,7 +5090,7 @@
         <v>14</v>
       </c>
       <c r="H134" t="s" s="2">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I134" t="s" s="2">
         <v>18</v>
@@ -5101,7 +5107,7 @@
         <v>14</v>
       </c>
       <c r="B135" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C135" t="s" s="2">
         <v>14</v>
@@ -5136,7 +5142,7 @@
         <v>14</v>
       </c>
       <c r="B136" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C136" t="s" s="2">
         <v>14</v>
@@ -5171,7 +5177,7 @@
         <v>14</v>
       </c>
       <c r="B137" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C137" t="s" s="2">
         <v>14</v>
@@ -5206,7 +5212,7 @@
         <v>14</v>
       </c>
       <c r="B138" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C138" t="s" s="2">
         <v>14</v>
@@ -5224,7 +5230,7 @@
         <v>14</v>
       </c>
       <c r="H138" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I138" t="s" s="2">
         <v>18</v>
@@ -5241,7 +5247,7 @@
         <v>14</v>
       </c>
       <c r="B139" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C139" t="s" s="2">
         <v>14</v>
@@ -5276,7 +5282,7 @@
         <v>14</v>
       </c>
       <c r="B140" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C140" t="s" s="2">
         <v>14</v>
@@ -5294,7 +5300,7 @@
         <v>14</v>
       </c>
       <c r="H140" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I140" t="s" s="2">
         <v>18</v>
@@ -5311,7 +5317,7 @@
         <v>14</v>
       </c>
       <c r="B141" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C141" t="s" s="2">
         <v>14</v>
@@ -5329,7 +5335,7 @@
         <v>14</v>
       </c>
       <c r="H141" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I141" t="s" s="2">
         <v>18</v>
@@ -5346,7 +5352,7 @@
         <v>14</v>
       </c>
       <c r="B142" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C142" t="s" s="2">
         <v>14</v>
@@ -5381,7 +5387,7 @@
         <v>14</v>
       </c>
       <c r="B143" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C143" t="s" s="2">
         <v>14</v>
@@ -5399,7 +5405,7 @@
         <v>14</v>
       </c>
       <c r="H143" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I143" t="s" s="2">
         <v>18</v>
@@ -5416,7 +5422,7 @@
         <v>14</v>
       </c>
       <c r="B144" t="s" s="2">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C144" t="s" s="2">
         <v>14</v>
@@ -5448,13 +5454,13 @@
     </row>
     <row r="145">
       <c r="A145" t="s" s="2">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="B145" t="s" s="2">
         <v>59</v>
       </c>
       <c r="C145" t="s" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D145" t="s" s="2">
         <v>14</v>
@@ -5463,13 +5469,13 @@
         <v>14</v>
       </c>
       <c r="F145" t="s" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G145" t="s" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H145" t="s" s="2">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I145" t="s" s="2">
         <v>18</v>
@@ -5539,7 +5545,7 @@
         <v>14</v>
       </c>
       <c r="H147" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I147" t="s" s="2">
         <v>18</v>
@@ -5679,7 +5685,7 @@
         <v>14</v>
       </c>
       <c r="H151" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I151" t="s" s="2">
         <v>18</v>
@@ -5728,13 +5734,13 @@
     </row>
     <row r="153">
       <c r="A153" t="s" s="2">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="B153" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C153" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D153" t="s" s="2">
         <v>14</v>
@@ -5743,13 +5749,13 @@
         <v>14</v>
       </c>
       <c r="F153" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G153" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H153" t="s" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I153" t="s" s="2">
         <v>18</v>
@@ -5766,7 +5772,7 @@
         <v>14</v>
       </c>
       <c r="B154" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C154" t="s" s="2">
         <v>14</v>
@@ -5801,7 +5807,7 @@
         <v>14</v>
       </c>
       <c r="B155" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C155" t="s" s="2">
         <v>14</v>
@@ -5836,7 +5842,7 @@
         <v>14</v>
       </c>
       <c r="B156" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C156" t="s" s="2">
         <v>14</v>
@@ -5871,7 +5877,7 @@
         <v>14</v>
       </c>
       <c r="B157" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C157" t="s" s="2">
         <v>14</v>
@@ -5906,7 +5912,7 @@
         <v>14</v>
       </c>
       <c r="B158" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C158" t="s" s="2">
         <v>14</v>
@@ -5941,7 +5947,7 @@
         <v>14</v>
       </c>
       <c r="B159" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C159" t="s" s="2">
         <v>14</v>
@@ -5976,7 +5982,7 @@
         <v>14</v>
       </c>
       <c r="B160" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C160" t="s" s="2">
         <v>14</v>
@@ -5994,7 +6000,7 @@
         <v>14</v>
       </c>
       <c r="H160" t="s" s="2">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I160" t="s" s="2">
         <v>18</v>
@@ -6011,7 +6017,7 @@
         <v>14</v>
       </c>
       <c r="B161" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C161" t="s" s="2">
         <v>14</v>
@@ -6029,7 +6035,7 @@
         <v>14</v>
       </c>
       <c r="H161" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I161" t="s" s="2">
         <v>18</v>
@@ -6046,7 +6052,7 @@
         <v>14</v>
       </c>
       <c r="B162" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C162" t="s" s="2">
         <v>14</v>
@@ -6064,7 +6070,7 @@
         <v>14</v>
       </c>
       <c r="H162" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I162" t="s" s="2">
         <v>18</v>
@@ -6081,7 +6087,7 @@
         <v>14</v>
       </c>
       <c r="B163" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C163" t="s" s="2">
         <v>14</v>
@@ -6099,7 +6105,7 @@
         <v>14</v>
       </c>
       <c r="H163" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I163" t="s" s="2">
         <v>18</v>
@@ -6116,7 +6122,7 @@
         <v>14</v>
       </c>
       <c r="B164" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C164" t="s" s="2">
         <v>14</v>
@@ -6134,7 +6140,7 @@
         <v>14</v>
       </c>
       <c r="H164" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I164" t="s" s="2">
         <v>18</v>
@@ -6151,7 +6157,7 @@
         <v>14</v>
       </c>
       <c r="B165" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C165" t="s" s="2">
         <v>14</v>
@@ -6169,7 +6175,7 @@
         <v>14</v>
       </c>
       <c r="H165" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I165" t="s" s="2">
         <v>18</v>
@@ -6186,7 +6192,7 @@
         <v>14</v>
       </c>
       <c r="B166" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C166" t="s" s="2">
         <v>14</v>
@@ -6221,7 +6227,7 @@
         <v>14</v>
       </c>
       <c r="B167" t="s" s="2">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C167" t="s" s="2">
         <v>14</v>
@@ -6253,13 +6259,13 @@
     </row>
     <row r="168">
       <c r="A168" t="s" s="2">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="B168" t="s" s="2">
         <v>61</v>
       </c>
       <c r="C168" t="s" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D168" t="s" s="2">
         <v>14</v>
@@ -6268,13 +6274,13 @@
         <v>14</v>
       </c>
       <c r="F168" t="s" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G168" t="s" s="2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H168" t="s" s="2">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I168" t="s" s="2">
         <v>18</v>
@@ -6309,7 +6315,7 @@
         <v>14</v>
       </c>
       <c r="H169" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I169" t="s" s="2">
         <v>18</v>
@@ -6344,7 +6350,7 @@
         <v>14</v>
       </c>
       <c r="H170" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I170" t="s" s="2">
         <v>18</v>
@@ -6379,7 +6385,7 @@
         <v>14</v>
       </c>
       <c r="H171" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I171" t="s" s="2">
         <v>18</v>
@@ -6414,7 +6420,7 @@
         <v>14</v>
       </c>
       <c r="H172" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I172" t="s" s="2">
         <v>18</v>
@@ -6449,7 +6455,7 @@
         <v>14</v>
       </c>
       <c r="H173" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I173" t="s" s="2">
         <v>18</v>
@@ -6533,13 +6539,13 @@
     </row>
     <row r="176">
       <c r="A176" t="s" s="2">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="B176" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C176" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D176" t="s" s="2">
         <v>14</v>
@@ -6548,13 +6554,13 @@
         <v>14</v>
       </c>
       <c r="F176" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G176" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H176" t="s" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I176" t="s" s="2">
         <v>18</v>
@@ -6571,7 +6577,7 @@
         <v>14</v>
       </c>
       <c r="B177" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C177" t="s" s="2">
         <v>14</v>
@@ -6606,7 +6612,7 @@
         <v>14</v>
       </c>
       <c r="B178" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C178" t="s" s="2">
         <v>14</v>
@@ -6641,7 +6647,7 @@
         <v>14</v>
       </c>
       <c r="B179" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C179" t="s" s="2">
         <v>14</v>
@@ -6676,7 +6682,7 @@
         <v>14</v>
       </c>
       <c r="B180" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C180" t="s" s="2">
         <v>14</v>
@@ -6711,7 +6717,7 @@
         <v>14</v>
       </c>
       <c r="B181" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C181" t="s" s="2">
         <v>14</v>
@@ -6746,7 +6752,7 @@
         <v>14</v>
       </c>
       <c r="B182" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C182" t="s" s="2">
         <v>14</v>
@@ -6781,7 +6787,7 @@
         <v>14</v>
       </c>
       <c r="B183" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C183" t="s" s="2">
         <v>14</v>
@@ -6816,7 +6822,7 @@
         <v>14</v>
       </c>
       <c r="B184" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C184" t="s" s="2">
         <v>14</v>
@@ -6851,7 +6857,7 @@
         <v>14</v>
       </c>
       <c r="B185" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C185" t="s" s="2">
         <v>14</v>
@@ -6886,7 +6892,7 @@
         <v>14</v>
       </c>
       <c r="B186" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C186" t="s" s="2">
         <v>14</v>
@@ -6904,7 +6910,7 @@
         <v>14</v>
       </c>
       <c r="H186" t="s" s="2">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="I186" t="s" s="2">
         <v>18</v>
@@ -6921,7 +6927,7 @@
         <v>14</v>
       </c>
       <c r="B187" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C187" t="s" s="2">
         <v>14</v>
@@ -6956,7 +6962,7 @@
         <v>14</v>
       </c>
       <c r="B188" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C188" t="s" s="2">
         <v>14</v>
@@ -6991,7 +6997,7 @@
         <v>14</v>
       </c>
       <c r="B189" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C189" t="s" s="2">
         <v>14</v>
@@ -7026,7 +7032,7 @@
         <v>14</v>
       </c>
       <c r="B190" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C190" t="s" s="2">
         <v>14</v>
@@ -7061,7 +7067,7 @@
         <v>14</v>
       </c>
       <c r="B191" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C191" t="s" s="2">
         <v>14</v>
@@ -7079,7 +7085,7 @@
         <v>14</v>
       </c>
       <c r="H191" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I191" t="s" s="2">
         <v>18</v>
@@ -7096,7 +7102,7 @@
         <v>14</v>
       </c>
       <c r="B192" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C192" t="s" s="2">
         <v>14</v>
@@ -7114,7 +7120,7 @@
         <v>14</v>
       </c>
       <c r="H192" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I192" t="s" s="2">
         <v>18</v>
@@ -7131,7 +7137,7 @@
         <v>14</v>
       </c>
       <c r="B193" t="s" s="2">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C193" t="s" s="2">
         <v>14</v>
@@ -7149,7 +7155,7 @@
         <v>14</v>
       </c>
       <c r="H193" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I193" t="s" s="2">
         <v>18</v>
@@ -7163,28 +7169,28 @@
     </row>
     <row r="194">
       <c r="A194" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="B194" t="s" s="2">
         <v>63</v>
       </c>
-      <c r="B194" t="s" s="2">
+      <c r="C194" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="D194" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="E194" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="F194" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="G194" t="s" s="2">
+        <v>14</v>
+      </c>
+      <c r="H194" t="s" s="2">
         <v>64</v>
-      </c>
-      <c r="C194" t="s" s="2">
-        <v>13</v>
-      </c>
-      <c r="D194" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="E194" t="s" s="2">
-        <v>14</v>
-      </c>
-      <c r="F194" t="s" s="2">
-        <v>15</v>
-      </c>
-      <c r="G194" t="s" s="2">
-        <v>16</v>
-      </c>
-      <c r="H194" t="s" s="2">
-        <v>29</v>
       </c>
       <c r="I194" t="s" s="2">
         <v>18</v>
@@ -7201,7 +7207,7 @@
         <v>14</v>
       </c>
       <c r="B195" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C195" t="s" s="2">
         <v>14</v>
@@ -7236,7 +7242,7 @@
         <v>14</v>
       </c>
       <c r="B196" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C196" t="s" s="2">
         <v>14</v>
@@ -7254,7 +7260,7 @@
         <v>14</v>
       </c>
       <c r="H196" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I196" t="s" s="2">
         <v>18</v>
@@ -7271,7 +7277,7 @@
         <v>14</v>
       </c>
       <c r="B197" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C197" t="s" s="2">
         <v>14</v>
@@ -7306,7 +7312,7 @@
         <v>14</v>
       </c>
       <c r="B198" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C198" t="s" s="2">
         <v>14</v>
@@ -7324,7 +7330,7 @@
         <v>14</v>
       </c>
       <c r="H198" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I198" t="s" s="2">
         <v>18</v>
@@ -7341,7 +7347,7 @@
         <v>14</v>
       </c>
       <c r="B199" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C199" t="s" s="2">
         <v>14</v>
@@ -7359,7 +7365,7 @@
         <v>14</v>
       </c>
       <c r="H199" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I199" t="s" s="2">
         <v>18</v>
@@ -7376,7 +7382,7 @@
         <v>14</v>
       </c>
       <c r="B200" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C200" t="s" s="2">
         <v>14</v>
@@ -7411,7 +7417,7 @@
         <v>14</v>
       </c>
       <c r="B201" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C201" t="s" s="2">
         <v>14</v>
@@ -7429,7 +7435,7 @@
         <v>14</v>
       </c>
       <c r="H201" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I201" t="s" s="2">
         <v>18</v>
@@ -7443,13 +7449,13 @@
     </row>
     <row r="202">
       <c r="A202" t="s" s="2">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="B202" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C202" t="s" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D202" t="s" s="2">
         <v>14</v>
@@ -7458,13 +7464,13 @@
         <v>14</v>
       </c>
       <c r="F202" t="s" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G202" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H202" t="s" s="2">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="I202" t="s" s="2">
         <v>18</v>
@@ -7481,7 +7487,7 @@
         <v>14</v>
       </c>
       <c r="B203" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C203" t="s" s="2">
         <v>14</v>
@@ -7499,7 +7505,7 @@
         <v>14</v>
       </c>
       <c r="H203" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I203" t="s" s="2">
         <v>18</v>
@@ -7516,7 +7522,7 @@
         <v>14</v>
       </c>
       <c r="B204" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C204" t="s" s="2">
         <v>14</v>
@@ -7534,7 +7540,7 @@
         <v>14</v>
       </c>
       <c r="H204" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I204" t="s" s="2">
         <v>18</v>
@@ -7551,7 +7557,7 @@
         <v>14</v>
       </c>
       <c r="B205" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C205" t="s" s="2">
         <v>14</v>
@@ -7586,7 +7592,7 @@
         <v>14</v>
       </c>
       <c r="B206" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C206" t="s" s="2">
         <v>14</v>
@@ -7604,7 +7610,7 @@
         <v>14</v>
       </c>
       <c r="H206" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I206" t="s" s="2">
         <v>18</v>
@@ -7621,7 +7627,7 @@
         <v>14</v>
       </c>
       <c r="B207" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C207" t="s" s="2">
         <v>14</v>
@@ -7656,7 +7662,7 @@
         <v>14</v>
       </c>
       <c r="B208" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C208" t="s" s="2">
         <v>14</v>
@@ -7674,7 +7680,7 @@
         <v>14</v>
       </c>
       <c r="H208" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I208" t="s" s="2">
         <v>18</v>
@@ -7691,7 +7697,7 @@
         <v>14</v>
       </c>
       <c r="B209" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C209" t="s" s="2">
         <v>14</v>
@@ -7726,7 +7732,7 @@
         <v>14</v>
       </c>
       <c r="B210" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C210" t="s" s="2">
         <v>14</v>
@@ -7744,7 +7750,7 @@
         <v>14</v>
       </c>
       <c r="H210" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I210" t="s" s="2">
         <v>18</v>
@@ -7761,7 +7767,7 @@
         <v>14</v>
       </c>
       <c r="B211" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C211" t="s" s="2">
         <v>14</v>
@@ -7779,7 +7785,7 @@
         <v>14</v>
       </c>
       <c r="H211" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I211" t="s" s="2">
         <v>18</v>
@@ -7796,7 +7802,7 @@
         <v>14</v>
       </c>
       <c r="B212" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C212" t="s" s="2">
         <v>14</v>
@@ -7831,7 +7837,7 @@
         <v>14</v>
       </c>
       <c r="B213" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C213" t="s" s="2">
         <v>14</v>
@@ -7849,7 +7855,7 @@
         <v>14</v>
       </c>
       <c r="H213" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I213" t="s" s="2">
         <v>18</v>
@@ -7866,7 +7872,7 @@
         <v>14</v>
       </c>
       <c r="B214" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C214" t="s" s="2">
         <v>14</v>
@@ -7884,7 +7890,7 @@
         <v>14</v>
       </c>
       <c r="H214" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I214" t="s" s="2">
         <v>18</v>
@@ -7901,7 +7907,7 @@
         <v>14</v>
       </c>
       <c r="B215" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C215" t="s" s="2">
         <v>14</v>
@@ -7919,7 +7925,7 @@
         <v>14</v>
       </c>
       <c r="H215" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I215" t="s" s="2">
         <v>18</v>
@@ -7936,7 +7942,7 @@
         <v>14</v>
       </c>
       <c r="B216" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C216" t="s" s="2">
         <v>14</v>
@@ -7971,7 +7977,7 @@
         <v>14</v>
       </c>
       <c r="B217" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C217" t="s" s="2">
         <v>14</v>
@@ -7989,7 +7995,7 @@
         <v>14</v>
       </c>
       <c r="H217" t="s" s="2">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I217" t="s" s="2">
         <v>18</v>
@@ -8006,7 +8012,7 @@
         <v>14</v>
       </c>
       <c r="B218" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C218" t="s" s="2">
         <v>14</v>
@@ -8024,7 +8030,7 @@
         <v>14</v>
       </c>
       <c r="H218" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I218" t="s" s="2">
         <v>18</v>
@@ -8041,7 +8047,7 @@
         <v>14</v>
       </c>
       <c r="B219" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C219" t="s" s="2">
         <v>14</v>
@@ -8059,7 +8065,7 @@
         <v>14</v>
       </c>
       <c r="H219" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I219" t="s" s="2">
         <v>18</v>
@@ -8076,7 +8082,7 @@
         <v>14</v>
       </c>
       <c r="B220" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C220" t="s" s="2">
         <v>14</v>
@@ -8094,7 +8100,7 @@
         <v>14</v>
       </c>
       <c r="H220" t="s" s="2">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I220" t="s" s="2">
         <v>18</v>
@@ -8111,7 +8117,7 @@
         <v>14</v>
       </c>
       <c r="B221" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C221" t="s" s="2">
         <v>14</v>
@@ -8129,7 +8135,7 @@
         <v>14</v>
       </c>
       <c r="H221" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I221" t="s" s="2">
         <v>18</v>
@@ -8146,7 +8152,7 @@
         <v>14</v>
       </c>
       <c r="B222" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C222" t="s" s="2">
         <v>14</v>
@@ -8164,7 +8170,7 @@
         <v>14</v>
       </c>
       <c r="H222" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I222" t="s" s="2">
         <v>18</v>
@@ -8181,7 +8187,7 @@
         <v>14</v>
       </c>
       <c r="B223" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C223" t="s" s="2">
         <v>14</v>
@@ -8199,7 +8205,7 @@
         <v>14</v>
       </c>
       <c r="H223" t="s" s="2">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="I223" t="s" s="2">
         <v>18</v>
@@ -8216,7 +8222,7 @@
         <v>14</v>
       </c>
       <c r="B224" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C224" t="s" s="2">
         <v>14</v>
@@ -8234,7 +8240,7 @@
         <v>14</v>
       </c>
       <c r="H224" t="s" s="2">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="I224" t="s" s="2">
         <v>18</v>
@@ -8251,7 +8257,7 @@
         <v>14</v>
       </c>
       <c r="B225" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C225" t="s" s="2">
         <v>14</v>
@@ -8286,7 +8292,7 @@
         <v>14</v>
       </c>
       <c r="B226" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C226" t="s" s="2">
         <v>14</v>
@@ -8321,7 +8327,7 @@
         <v>14</v>
       </c>
       <c r="B227" t="s" s="2">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C227" t="s" s="2">
         <v>14</v>
@@ -8353,10 +8359,10 @@
     </row>
     <row r="228">
       <c r="A228" t="s" s="2">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B228" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C228" t="s" s="2">
         <v>13</v>
@@ -8391,7 +8397,7 @@
         <v>14</v>
       </c>
       <c r="B229" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C229" t="s" s="2">
         <v>14</v>
@@ -8426,7 +8432,7 @@
         <v>14</v>
       </c>
       <c r="B230" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C230" t="s" s="2">
         <v>14</v>
@@ -8461,7 +8467,7 @@
         <v>14</v>
       </c>
       <c r="B231" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C231" t="s" s="2">
         <v>14</v>
@@ -8496,7 +8502,7 @@
         <v>14</v>
       </c>
       <c r="B232" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C232" t="s" s="2">
         <v>14</v>
@@ -8531,7 +8537,7 @@
         <v>14</v>
       </c>
       <c r="B233" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C233" t="s" s="2">
         <v>14</v>
@@ -8566,7 +8572,7 @@
         <v>14</v>
       </c>
       <c r="B234" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C234" t="s" s="2">
         <v>14</v>
@@ -8601,7 +8607,7 @@
         <v>14</v>
       </c>
       <c r="B235" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C235" t="s" s="2">
         <v>14</v>
@@ -8636,7 +8642,7 @@
         <v>14</v>
       </c>
       <c r="B236" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C236" t="s" s="2">
         <v>14</v>
@@ -8671,7 +8677,7 @@
         <v>14</v>
       </c>
       <c r="B237" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C237" t="s" s="2">
         <v>14</v>
@@ -8706,7 +8712,7 @@
         <v>14</v>
       </c>
       <c r="B238" t="s" s="2">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C238" t="s" s="2">
         <v>14</v>
@@ -8738,10 +8744,10 @@
     </row>
     <row r="239">
       <c r="A239" t="s" s="2">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B239" t="s" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C239" t="s" s="2">
         <v>13</v>
@@ -8759,7 +8765,7 @@
         <v>21</v>
       </c>
       <c r="H239" t="s" s="2">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I239" t="s" s="2">
         <v>18</v>
@@ -8776,7 +8782,7 @@
         <v>14</v>
       </c>
       <c r="B240" t="s" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C240" t="s" s="2">
         <v>14</v>
@@ -8811,7 +8817,7 @@
         <v>14</v>
       </c>
       <c r="B241" t="s" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C241" t="s" s="2">
         <v>14</v>
@@ -8846,7 +8852,7 @@
         <v>14</v>
       </c>
       <c r="B242" t="s" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C242" t="s" s="2">
         <v>14</v>
@@ -8881,7 +8887,7 @@
         <v>14</v>
       </c>
       <c r="B243" t="s" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C243" t="s" s="2">
         <v>14</v>
@@ -8916,7 +8922,7 @@
         <v>14</v>
       </c>
       <c r="B244" t="s" s="2">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C244" t="s" s="2">
         <v>14</v>
@@ -8934,7 +8940,7 @@
         <v>14</v>
       </c>
       <c r="H244" t="s" s="2">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I244" t="s" s="2">
         <v>18</v>
@@ -8948,10 +8954,10 @@
     </row>
     <row r="245">
       <c r="A245" t="s" s="2">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B245" t="s" s="2">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C245" t="s" s="2">
         <v>13</v>
@@ -8983,10 +8989,10 @@
     </row>
     <row r="246">
       <c r="A246" t="s" s="2">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B246" t="s" s="2">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C246" t="s" s="2">
         <v>13</v>
@@ -9021,7 +9027,7 @@
         <v>14</v>
       </c>
       <c r="B247" t="s" s="2">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C247" t="s" s="2">
         <v>14</v>
@@ -9056,7 +9062,7 @@
         <v>14</v>
       </c>
       <c r="B248" t="s" s="2">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C248" t="s" s="2">
         <v>14</v>
@@ -9088,10 +9094,10 @@
     </row>
     <row r="249">
       <c r="A249" t="s" s="2">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B249" t="s" s="2">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C249" t="s" s="2">
         <v>13</v>
@@ -9126,7 +9132,7 @@
         <v>14</v>
       </c>
       <c r="B250" t="s" s="2">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C250" t="s" s="2">
         <v>14</v>
@@ -9161,7 +9167,7 @@
         <v>14</v>
       </c>
       <c r="B251" t="s" s="2">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C251" t="s" s="2">
         <v>14</v>
@@ -9193,10 +9199,10 @@
     </row>
     <row r="252">
       <c r="A252" t="s" s="2">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B252" t="s" s="2">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C252" t="s" s="2">
         <v>13</v>
@@ -9214,7 +9220,7 @@
         <v>16</v>
       </c>
       <c r="H252" t="s" s="2">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I252" t="s" s="2">
         <v>18</v>
@@ -9231,7 +9237,7 @@
         <v>14</v>
       </c>
       <c r="B253" t="s" s="2">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C253" t="s" s="2">
         <v>14</v>
@@ -9263,10 +9269,10 @@
     </row>
     <row r="254">
       <c r="A254" t="s" s="2">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B254" t="s" s="2">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C254" t="s" s="2">
         <v>13</v>
@@ -9298,10 +9304,10 @@
     </row>
     <row r="255">
       <c r="A255" t="s" s="2">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B255" t="s" s="2">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C255" t="s" s="2">
         <v>13</v>
@@ -9316,7 +9322,7 @@
         <v>15</v>
       </c>
       <c r="G255" t="s" s="2">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H255" t="s" s="2">
         <v>14</v>
@@ -9333,10 +9339,10 @@
     </row>
     <row r="256">
       <c r="A256" t="s" s="2">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B256" t="s" s="2">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C256" t="s" s="2">
         <v>13</v>
@@ -9371,7 +9377,7 @@
         <v>14</v>
       </c>
       <c r="B257" t="s" s="2">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C257" t="s" s="2">
         <v>14</v>

</xml_diff>